<commit_message>
Stage 8 review fixes: A-020
</commit_message>
<xml_diff>
--- a/output/archive/VellacombeData/Clients/RC17/VD-25-066/Routes/Paused/RC17_storage_11Jun25.xlsx
+++ b/output/archive/VellacombeData/Clients/RC17/VD-25-066/Routes/Paused/RC17_storage_11Jun25.xlsx
@@ -148,7 +148,7 @@
   <commentList>
     <comment ref="G8" authorId="0" shapeId="0">
       <text>
-        <t>Desiccant needs changing before anyone opens this vial again.</t>
+        <t>Consult the storage inventory and compound cards before any reuse; do not infer identity or storage requirements from this summary.</t>
       </text>
     </comment>
   </commentList>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -574,136 +574,41 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Protected amine intermediate</t>
+          <t>Isolated intermediates</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Solid</t>
+          <t>See compound cards</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Controlled storage, cabinet 2</t>
+          <t>Controlled storage; see storage records</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Amber glass, screw cap</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>[TBC]</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>11 Jun 2025</t>
-        </is>
-      </c>
+          <t>See storage records</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Hygroscopic; keep desiccated</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Coupled ester intermediate</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Oil</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Controlled storage, cabinet 2</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Amber glass</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>11 Jun 2025</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr"/>
-    </row>
+          <t>Programme paused</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Chloro-pyrimidine intermediate</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Solid</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Controlled storage, cabinet 3</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Glass vial</t>
-        </is>
-      </c>
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Check seal before reuse</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Impurity reference, route B</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Solution in DMSO</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Freezer</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Screw-cap vial</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>[TBC] concentration</t>
-        </is>
-      </c>
-    </row>
-    <row r="12"/>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr"/>
-      <c r="B13" s="2" t="inlineStr"/>
-      <c r="C13" s="2" t="inlineStr"/>
-      <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -762,12 +667,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Route B confirmed on paper</t>
+          <t>Backup-route review</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Literature and conditions check</t>
+          <t>Consult route scout records</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -785,12 +690,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Protected amine re-characterised</t>
+          <t>Stored intermediates reviewed before reuse</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>1H NMR and HPLC</t>
+          <t>Check compound cards and storage records</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -808,12 +713,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Impurity standards prepared</t>
+          <t>Impurity-standard work</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Route B impurity set</t>
+          <t>Scope to be confirmed on restart</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">

</xml_diff>